<commit_message>
updated the script to show Sumar Registru Contracte updated the name from "Inexistente" in "Necorelate"
</commit_message>
<xml_diff>
--- a/extrase_pt_conta.xlsx
+++ b/extrase_pt_conta.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D159"/>
+  <dimension ref="A1:D166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1279,127 +1279,127 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>316</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>148799</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Proiectare Parc Pantelimon</t>
+          <t>PUZ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>08.05.2025</t>
+          <t>17.10.2023</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>436</t>
+          <t>422</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>149/167011</t>
+          <t>148799</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>proiectare si executie cladiri nZEB</t>
+          <t>Proiectare Parc Pantelimon</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>30.06.2025</t>
+          <t>08.05.2025</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>436</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>152515</t>
+          <t>149/167011</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>DALI, PT, AT Zona Inel II</t>
+          <t>proiectare si executie cladiri nZEB</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>02.08.2021</t>
+          <t>30.06.2025</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>365</t>
+          <t>199</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>152528</t>
+          <t>152515</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ST Pasaj Aurel Vlaicu</t>
+          <t>DALI, PT, AT Zona Inel II</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>30.08.2024</t>
+          <t>02.08.2021</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>295</t>
+          <t>365</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>15327</t>
+          <t>152528</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SF centru integrat de Mobilitate Urbana</t>
+          <t>ST Pasaj Aurel Vlaicu</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>06.06.2023</t>
+          <t>30.08.2024</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>294</t>
+          <t>295</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>15329</t>
+          <t>15327</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SF statii</t>
+          <t>SF centru integrat de Mobilitate Urbana</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1411,83 +1411,83 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>294</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>153782</t>
+          <t>15329</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>studii trafic</t>
+          <t>SF statii</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>07.08.2024</t>
+          <t>06.06.2023</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>282</t>
+          <t>362</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>15796</t>
+          <t>153782</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>MP ITS</t>
+          <t>studii trafic</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>06.04.2023</t>
+          <t>07.08.2024</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>375</t>
+          <t>282</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>160314</t>
+          <t>15796</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ACTUALIARE STUDIU TRAFIC</t>
+          <t>MP ITS</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>22.10.2024</t>
+          <t>06.04.2023</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>376</t>
+          <t>375</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>160318</t>
+          <t>160314</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ACTUALIZARE POAT MOBILITATE URBANA</t>
+          <t>ACTUALIARE STUDIU TRAFIC</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1499,17 +1499,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>376</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>160323</t>
+          <t>160318</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ACTUALIZARE POAT CARTIERE REZIDENTIALE</t>
+          <t>ACTUALIZARE POAT MOBILITATE URBANA</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1521,100 +1521,100 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>455</t>
+          <t>377</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>161/184449</t>
+          <t>160323</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>MP gradinita 269</t>
+          <t>ACTUALIZARE POAT CARTIERE REZIDENTIALE</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>28.08.2025</t>
+          <t>22.10.2024</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>205</t>
+          <t>455</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>162488</t>
+          <t>161/184449</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>DALI, PT HUB</t>
+          <t>MP gradinita 269</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>01.11.2021</t>
+          <t>28.08.2025</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>298</t>
+          <t>451</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>165/172800</t>
+          <t>16244</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Consulatanta si cerere finantare blocuri</t>
+          <t>SF DAMBU</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>22.06.2023</t>
+          <t>06.08.2025</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>299</t>
+          <t>205</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>166/172803</t>
+          <t>162488</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Consulatanta si cerere finantare blocuri</t>
+          <t>DALI, PT HUB</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>22.06.2023</t>
+          <t>01.11.2021</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>298</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>167/172807</t>
+          <t>165/172800</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1631,2286 +1631,2440 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>299</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>16779</t>
+          <t>166/172803</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>SF, PT TICKETING</t>
+          <t>Consulatanta si cerere finantare blocuri</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>13.02.2025</t>
+          <t>22.06.2023</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>493</t>
+          <t>300</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>168</t>
+          <t>167/172807</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>SF ITS INTEGRAT SMART GREEN MOBILITY</t>
+          <t>Consulatanta si cerere finantare blocuri</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>22.06.2023</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>301</t>
+          <t>404</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>168/172809</t>
+          <t>16779</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Consulatanta si cerere finantare blocuri</t>
+          <t>SF, PT TICKETING</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>22.06.2023</t>
+          <t>13.02.2025</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>495</t>
+          <t>493</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>168</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>DALI crestere siguranta rutiera</t>
+          <t>SF ITS INTEGRAT SMART GREEN MOBILITY</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>23.12.205</t>
+          <t>09.12.2025</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>368</t>
+          <t>301</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>170450</t>
+          <t>168/172809</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>100 orase</t>
+          <t>Consulatanta si cerere finantare blocuri</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>04.09.2024</t>
+          <t>22.06.2023</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>487</t>
+          <t>373</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>172/195966</t>
+          <t>16850</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Acord cadru, contract subsecvent 7 statii incarcare</t>
+          <t>DALI, PT Gradina Publica</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>14.10.2024</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>366</t>
+          <t>495</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>173/206845</t>
+          <t>169</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve"> SO SMART CITY</t>
+          <t>DALI crestere siguranta rutiera</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>30.08.2024</t>
+          <t>23.12.205</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>368</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>17611</t>
+          <t>170450</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Optimizare coridor Nord-Sud</t>
+          <t>100 orase</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>18.02.2022</t>
+          <t>04.09.2024</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>370</t>
+          <t>487</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>176240</t>
+          <t>172/195966</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>PIRU</t>
+          <t>Acord cadru, contract subsecvent 7 statii incarcare</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>03.10.2024</t>
+          <t>09.10.2025</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>317</t>
+          <t>366</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>182393</t>
+          <t>173/206845</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>SO Autobuze</t>
+          <t xml:space="preserve"> SO SMART CITY</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>20.10.2023</t>
+          <t>30.08.2024</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>225</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>187125</t>
+          <t>17611</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>SO Microbuze</t>
+          <t>Optimizare coridor Nord-Sud</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>27.10.2023</t>
+          <t>18.02.2022</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>482</t>
+          <t>370</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>176240</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>consultanta fonduri Strategic projects under the critical raw materials ac</t>
+          <t>PIRU</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>03.10.2024</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>477</t>
+          <t>317</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>191162</t>
+          <t>182393</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Consultanta management proiect Modernizare Depou de tramvaie etapa 1</t>
+          <t>SO Autobuze</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>13.10.2025</t>
+          <t>20.10.2023</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>344</t>
+          <t>320</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>19222</t>
+          <t>187125</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>PT Trafic Management</t>
+          <t>SO Microbuze</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>27.03.2024</t>
+          <t>27.10.2023</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>467</t>
+          <t>482</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>19281</t>
+          <t>189</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>CF PARAU DAMBU</t>
+          <t>consultanta fonduri Strategic projects under the critical raw materials ac</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>22.09.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>477</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>195-214286</t>
+          <t>191162</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Consultanta si AT finantari cladiri tip NZEB</t>
+          <t>Consultanta management proiect Modernizare Depou de tramvaie etapa 1</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>13.09.2022</t>
+          <t>13.10.2025</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>344</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>196577</t>
+          <t>19222</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SO platforma electronica</t>
+          <t>PT Trafic Management</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>13.11.2023</t>
+          <t>27.03.2024</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>438</t>
+          <t>467</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>19281</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SO delegare transport public</t>
+          <t>CF PARAU DAMBU</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>30.06.2025</t>
+          <t>22.09.2025</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>456</t>
+          <t>260</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>20134</t>
+          <t>195-214286</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Proiectare si asistenta tehnica autobaza</t>
+          <t>Consultanta si AT finantari cladiri tip NZEB</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>28.08.2025</t>
+          <t>13.09.2022</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>321</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2023/S 139-445422</t>
+          <t>196577</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>TICKETING</t>
+          <t>SO platforma electronica</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>11.12.2023</t>
+          <t>13.11.2023</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>383</t>
+          <t>438</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>203726</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>SF STATII INCARCARE</t>
+          <t>SO delegare transport public</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>23.10.2024</t>
+          <t>30.06.2025</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>483</t>
+          <t>456</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>205926</t>
+          <t>20134</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Consultanta management proiect Modernizare Depou de tramvaie etapa 2</t>
+          <t>Proiectare si asistenta tehnica autobaza</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>03.11.2025</t>
+          <t>28.08.2025</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>388</t>
+          <t>324</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>20616</t>
+          <t>2023/S 139-445422</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Cerere finantare</t>
+          <t>TICKETING</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>10.12.2024</t>
+          <t>11.12.2023</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>383</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>21012</t>
+          <t>203726</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>SO delegare transport public</t>
+          <t>SF STATII INCARCARE</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>05.12.2024</t>
+          <t>23.10.2024</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>269</t>
+          <t>483</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>212729</t>
+          <t>205926</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>SF parcari</t>
+          <t>Consultanta management proiect Modernizare Depou de tramvaie etapa 2</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>21.11.2022</t>
+          <t>03.11.2025</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>390</t>
+          <t>388</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>21295</t>
+          <t>20616</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Sf sistem informatic</t>
+          <t>Cerere finantare</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>20.12.2024</t>
+          <t>10.12.2024</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>296</t>
+          <t>400</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>21702</t>
+          <t>21012</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>SF ITS</t>
+          <t>SO delegare transport public</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>06.06.2023</t>
+          <t>05.12.2024</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>426</t>
+          <t>269</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>22237</t>
+          <t>212729</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>SO DELEGARE TP</t>
+          <t>SF parcari</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>26.05.2025</t>
+          <t>21.11.2022</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>395</t>
+          <t>390</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>225527</t>
+          <t>21295</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>MP HUB</t>
+          <t>Sf sistem informatic</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>23.12.2024</t>
+          <t>20.12.2024</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>392</t>
+          <t>296</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>227342</t>
+          <t>21702</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>PT si Ex CAV FAZA 1</t>
+          <t>SF ITS</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>30.12.2024</t>
+          <t>06.06.2023</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>285</t>
+          <t>426</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>22857</t>
+          <t>22237</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>SF Trafic Management</t>
+          <t>SO DELEGARE TP</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>08.05.2023</t>
+          <t>26.05.2025</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>478</t>
+          <t>395</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>23455</t>
+          <t>225527</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Consultanta program incluziune si demnitate sociala</t>
+          <t>MP HUB</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>28.08.2025</t>
+          <t>23.12.2024</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>446</t>
+          <t>392</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>227342</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Cerere finnatare</t>
+          <t>PT si Ex CAV FAZA 1</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>30.12.2024</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>292</t>
+          <t>285</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>23600</t>
+          <t>22857</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>MP achizitie autobuze</t>
+          <t>SF Trafic Management</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>29.05.2023</t>
+          <t>08.05.2023</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>475</t>
+          <t>478</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>23728</t>
+          <t>23455</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Consultanta infrastructura transport nemotorizat</t>
+          <t>Consultanta program incluziune si demnitate sociala</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>28.08.2025</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>312</t>
+          <t>446</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>241/200201</t>
+          <t>236</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Cereri finantare cladiri</t>
+          <t>Cerere finnatare</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>07.09.2023</t>
+          <t>17.07.2025</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>308</t>
+          <t>292</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>24633</t>
+          <t>23600</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>SF ITS Runda 1</t>
+          <t>MP achizitie autobuze</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>27.07.2023</t>
+          <t>29.05.2023</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>309</t>
+          <t>475</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>24634</t>
+          <t>23728</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>SF ITS Runda 2</t>
+          <t>Consultanta infrastructura transport nemotorizat</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>27.07.2023</t>
+          <t>02.09.2025</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>314</t>
+          <t>312</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>250/207060</t>
+          <t>241/200201</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>analiza DNSH</t>
+          <t>Cereri finantare cladiri</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>26.09.2023</t>
+          <t>07.09.2023</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>328</t>
+          <t>308</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2545</t>
+          <t>24633</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>SF modernizare TP</t>
+          <t>SF ITS Runda 1</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>02.02.2024</t>
+          <t>27.07.2023</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>327</t>
+          <t>309</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2550</t>
+          <t>24634</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>CF modernizare TP</t>
+          <t>SF ITS Runda 2</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>02.02.2024</t>
+          <t>27.07.2023</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>363</t>
+          <t>314</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>250/207060</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>SF sistem inteligent urban Reghin</t>
+          <t>analiza DNSH</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>08.08.2024</t>
+          <t>26.09.2023</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>340</t>
+          <t>328</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>27/151030</t>
+          <t>2545</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Analiza DNSH Gradinita 269</t>
+          <t>SF modernizare TP</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>20.03.2024</t>
+          <t>02.02.2024</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>327</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>28280</t>
+          <t>2550</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>SF sistem tranport ecologic</t>
+          <t>CF modernizare TP</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>01.08.2022</t>
+          <t>02.02.2024</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>313</t>
+          <t>363</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>284/134075</t>
+          <t>263</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>SF CAV mare</t>
+          <t>SF sistem inteligent urban Reghin</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>15.09.2023</t>
+          <t>08.08.2024</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>385</t>
+          <t>340</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>289178</t>
+          <t>27/151030</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>SO, ST</t>
+          <t>Analiza DNSH Gradinita 269</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>03.12.2024</t>
+          <t>20.03.2024</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>255</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2935</t>
+          <t>28280</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Consultanta expert cooptat</t>
+          <t>SF sistem tranport ecologic</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>05.02.2024</t>
+          <t>01.08.2022</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>359</t>
+          <t>313</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>29364</t>
+          <t>284/134075</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>PT, AT si Ex Modernizare parc auto</t>
+          <t>SF CAV mare</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>25.07.2024</t>
+          <t>15.09.2023</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>445</t>
+          <t>385</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>289178</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Proiectare si executie campus</t>
+          <t>SO, ST</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>07.07.2025</t>
+          <t>03.12.2024</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>447</t>
+          <t>329</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>30509</t>
+          <t>2935</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Proiectare autobaza</t>
+          <t>Consultanta expert cooptat</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>18.07.2025</t>
+          <t>05.02.2024</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>399</t>
+          <t>359</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>31/C</t>
+          <t>29364</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>DALI HVAC</t>
+          <t>PT, AT si Ex Modernizare parc auto</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>23.01.2025</t>
+          <t>25.07.2024</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>387</t>
+          <t>445</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>PT CAROL DAVILA</t>
+          <t>Proiectare si executie campus</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>06.12.2024</t>
+          <t>07.07.2025</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>289</t>
+          <t>447</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>31052</t>
+          <t>30509</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>SO achizitie autobuze</t>
+          <t>Proiectare autobaza</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>26.05.2023</t>
+          <t>18.07.2025</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>399</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>31252</t>
+          <t>31/C</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>ITS</t>
+          <t>DALI HVAC</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>06.08.2024</t>
+          <t>23.01.2025</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>484</t>
+          <t>387</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>31860</t>
+          <t>310</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Consultanta monument istoric Fortul 13 Jilava</t>
+          <t>PT CAROL DAVILA</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>06.12.2024</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>452</t>
+          <t>289</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>33289</t>
+          <t>31052</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>CF autobaza</t>
+          <t>SO achizitie autobuze</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>06.08.2025</t>
+          <t>26.05.2023</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>259</t>
+          <t>361</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>33887</t>
+          <t>31252</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>consultanta,SF,PT infrastructura transport verd-ITS</t>
+          <t>ITS</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>12.09.2022</t>
+          <t>06.08.2024</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>379</t>
+          <t>484</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>34023</t>
+          <t>31860</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>SF UMF</t>
+          <t>Consultanta monument istoric Fortul 13 Jilava</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>15.11.2024</t>
+          <t>05.11.2025</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>304</t>
+          <t>452</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>36674</t>
+          <t>33289</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>DALI pietonal</t>
+          <t>CF autobaza</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>12.07.2023</t>
+          <t>06.08.2025</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>311</t>
+          <t>259</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>37511</t>
+          <t>33887</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>MP Digitalizare TP etapa II</t>
+          <t>consultanta,SF,PT infrastructura transport verd-ITS</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>01.09.2023</t>
+          <t>12.09.2022</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>379</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>37907</t>
+          <t>34023</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>SF SI PT CORIDOR DE MOBILITATE POAT</t>
+          <t>SF UMF</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>06.10.2022</t>
+          <t>15.11.2024</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>416</t>
+          <t>304</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>37958</t>
+          <t>36674</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>PT, AT rest lucrari zona pietonala centrala</t>
+          <t>DALI pietonal</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>19.02.2025</t>
+          <t>12.07.2023</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>402</t>
+          <t>311</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>38629</t>
+          <t>37511</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ASISTENTA TEHNICA CONSULTARE PUBLICA POR INFRASTRUCTURA AGREMENT</t>
+          <t>MP Digitalizare TP etapa II</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>04.02.2025</t>
+          <t>01.09.2023</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>263</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>38921</t>
+          <t>37907</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>ASISTENTA TEHNICA CONSULTARE PUBLICA POR ZONE URBANE</t>
+          <t>SF SI PT CORIDOR DE MOBILITATE POAT</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>04.02.2025</t>
+          <t>06.10.2022</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>315</t>
+          <t>416</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>41693</t>
+          <t>37958</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ITS etapa 2</t>
+          <t>PT, AT rest lucrari zona pietonala centrala</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>28.09.2023</t>
+          <t>19.02.2025</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>406</t>
+          <t>402</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>41721</t>
+          <t>38629</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>CF Achizitie autobuze</t>
+          <t>ASISTENTA TEHNICA CONSULTARE PUBLICA POR INFRASTRUCTURA AGREMENT</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>25.02.2025</t>
+          <t>04.02.2025</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>441</t>
+          <t>401</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>4201</t>
+          <t>38921</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Proiectare si asistenta tehnica trafic management</t>
+          <t>ASISTENTA TEHNICA CONSULTARE PUBLICA POR ZONE URBANE</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>07.07.2025</t>
+          <t>04.02.2025</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>315</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>43577</t>
+          <t>41693</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Asistenta tehnica achizitie autobuze</t>
+          <t>ITS etapa 2</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>16.06.2020</t>
+          <t>28.09.2023</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>406</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>47/37457</t>
+          <t>41721</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>SF CAV</t>
+          <t>CF Achizitie autobuze</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>13.03.2023</t>
+          <t>25.02.2025</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>407</t>
+          <t>441</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>4754</t>
+          <t>4201</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Proiectare, asistenta si furnizare Centru integrat de mobilitate urbana ITS</t>
+          <t>Proiectare si asistenta tehnica trafic management</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>27.02.2025</t>
+          <t>07.07.2025</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>275</t>
+          <t>152</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>4795</t>
+          <t>43577</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Consultanta PNRR C15</t>
+          <t>Asistenta tehnica achizitie autobuze</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>21.02.2023</t>
+          <t>16.06.2020</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>417</t>
+          <t>408</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>48 145223</t>
+          <t>43683</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Consultanta cladiri Bauhaus Inst Pneuftiziologie Marius Nasta - corp nou</t>
+          <t>Acting Together for Green Cities-identificare zone , planuri conceptuale</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>09.04.2025</t>
+          <t>26.02.2026</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>346</t>
+          <t>278</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>51/158930</t>
+          <t>47/37457</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Dotari scoli</t>
+          <t>SF CAV</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>08.04.2024</t>
+          <t>13.03.2023</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>338.1</t>
+          <t>407</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>5233</t>
+          <t>4754</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>SIDU</t>
+          <t>Proiectare, asistenta si furnizare Centru integrat de mobilitate urbana ITS</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>05.03.2024</t>
+          <t>27.02.2025</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>275</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>54043</t>
+          <t>4795</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Consultanta achiziie autobuze</t>
+          <t>Consultanta PNRR C15</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>17.03.2023</t>
+          <t>21.02.2023</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>434</t>
+          <t>417</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>48 145223</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Expertiza tehnica si DALI sediul administratiei C1-C6</t>
+          <t>Consultanta cladiri Bauhaus Inst Pneuftiziologie Marius Nasta - corp nou</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>09.04.2025</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>398</t>
+          <t>346</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>5971</t>
+          <t>51/158930</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>SO ticketing</t>
+          <t>Dotari scoli</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>21.01.2025</t>
+          <t>08.04.2024</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>274</t>
+          <t>338.1</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>5975</t>
+          <t>5233</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Consultanta</t>
+          <t>SIDU</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>15.02.2023</t>
+          <t>05.03.2024</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>281</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>643</t>
+          <t>54043</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Proiectare si consultanta accesare fonduri terminal intermodal port</t>
+          <t>Consultanta achiziie autobuze</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>10.02.2025</t>
+          <t>17.03.2023</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>427</t>
+          <t>434</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>66326</t>
+          <t>58</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>SF Dezvoltare sistem management urban</t>
+          <t>Expertiza tehnica si DALI sediul administratiei C1-C6</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>05.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>398</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>6873</t>
+          <t>5971</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Spitalul Horezu</t>
+          <t>SO ticketing</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>01.08.2024</t>
+          <t>21.01.2025</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>277</t>
+          <t>274</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>7025</t>
+          <t>5975</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>MP modernizare transport public prin achizitie de autobuze oras Bucecea</t>
+          <t>Consultanta</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>13.03.2023</t>
+          <t>15.02.2023</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>347</t>
+          <t>403</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>76263</t>
+          <t>643</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>SF Air City</t>
+          <t>Proiectare si consultanta accesare fonduri terminal intermodal port</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>19.04.2024</t>
+          <t>10.02.2025</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>412</t>
+          <t>427</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>7955</t>
+          <t>66326</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>DALI Gradina publica si parcare</t>
+          <t>SF Dezvoltare sistem management urban</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>16.01.2025</t>
+          <t>05.06.2025</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>420</t>
+          <t>360</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>80/149560</t>
+          <t>6873</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Acord subsecvent 2 la acord cadru 137516 - modernizare sistem rutier, scoala 103 si 126</t>
+          <t>Spitalul Horezu</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>29.04.2025</t>
+          <t>01.08.2024</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>277</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>80145</t>
+          <t>7025</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Consultanta E-Ticketing</t>
+          <t>MP modernizare transport public prin achizitie de autobuze oras Bucecea</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>12.08.2020</t>
+          <t>13.03.2023</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>276</t>
+          <t>347</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>8121</t>
+          <t>76263</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t xml:space="preserve">MP Proiectare sistem inteligent de planificare a calatoriilor cu transportul public </t>
+          <t>SF Air City</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>01.03.2023</t>
+          <t>19.04.2024</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>319</t>
+          <t>412</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>839</t>
+          <t>7955</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>SF ITS statii</t>
+          <t>DALI Gradina publica si parcare</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>27.10.2023</t>
+          <t>16.01.2025</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>439</t>
+          <t>420</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>80/149560</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>SO Achizitie autobuze</t>
+          <t>Acord subsecvent 2 la acord cadru 137516 - modernizare sistem rutier, scoala 103 si 126</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>04.07.2025</t>
+          <t>29.04.2025</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>440</t>
+          <t>156</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>80145</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>SF Autobaza</t>
+          <t>Consultanta E-Ticketing</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>04.07.2025</t>
+          <t>12.08.2020</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>276</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>8810</t>
+          <t>8121</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Consultanta PNRR</t>
+          <t xml:space="preserve">MP Proiectare sistem inteligent de planificare a calatoriilor cu transportul public </t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>08.03.2022</t>
+          <t>01.03.2023</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>462</t>
+          <t>319</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>8869</t>
+          <t>839</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>SF cu elemente DALI constructii civile programe screening</t>
+          <t>SF ITS statii</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>05.09.2025</t>
+          <t>27.10.2023</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>389</t>
+          <t>439</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>8887</t>
+          <t>87</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Studiu de obstacolare</t>
+          <t>SO Achizitie autobuze</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>17.12.2024</t>
+          <t>04.07.2025</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>474</t>
+          <t>440</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>91656</t>
+          <t>88</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>SO fundamentare centru comercial, parcari</t>
+          <t>SF Autobaza</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>02.10.2025</t>
+          <t>04.07.2025</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>413</t>
+          <t>232</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>99283</t>
+          <t>8810</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Consultanta regenerare urbana</t>
+          <t>Consultanta PNRR</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>20.03.2025</t>
+          <t>08.03.2022</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>423</t>
+          <t>462</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>9940</t>
+          <t>8869</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>SF, DTAC, DTOE centru ingrijiri paleative</t>
+          <t>SF cu elemente DALI constructii civile programe screening</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>12.05.2025</t>
+          <t>05.09.2025</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>337</t>
+          <t>389</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>CDSF02261</t>
+          <t>8887</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>ST Planseu unirii</t>
+          <t>Studiu de obstacolare</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>26.02.2024</t>
+          <t>17.12.2024</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>348</t>
+          <t>474</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>CDSF04301</t>
+          <t>91656</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Pasaj Unirii PT, AT planseu Dambovita</t>
+          <t>SO fundamentare centru comercial, parcari</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>30.04.2024</t>
+          <t>02.10.2025</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>349</t>
+          <t>473</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>CDSF0508_</t>
+          <t>91670</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Pasaj Unirii Studiu Trafic</t>
+          <t>DALI zona Parc Teatru</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>30.04.2024</t>
+          <t>02.10.2025</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>476</t>
+          <t>394</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>CDSF0903</t>
+          <t>96</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>CF gradinita 242</t>
+          <t>DALI RADU BELLER</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>03.09.2025</t>
+          <t>30.12.2024</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>458</t>
+          <t>490</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>J-AC 271</t>
+          <t>98726</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>DALI Cresterea sigurantei rutiere cartier Bucurestii Noi</t>
+          <t>DALI ZONA CENTRALA</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>09.09.2025</t>
+          <t>22.10.2025</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>459</t>
+          <t>413</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>J-AC 272</t>
+          <t>99283</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>DALI Cresterea sigurantei rutiere cartier Piata Romana</t>
+          <t>Consultanta regenerare urbana</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>09.09.2025</t>
+          <t>20.03.2025</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>460</t>
+          <t>423</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>J-AC 273</t>
+          <t>9940</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>DALI Cresterea sigurantei rutiere cartier Grivita</t>
+          <t>SF, DTAC, DTOE centru ingrijiri paleative</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>09.09.2025</t>
+          <t>12.05.2025</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
+          <t>337</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>CDSF02261</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>ST Planseu unirii</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>26.02.2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>348</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>CDSF04301</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Pasaj Unirii PT, AT planseu Dambovita</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>30.04.2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>349</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>CDSF0508_</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Pasaj Unirii Studiu Trafic</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>30.04.2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>476</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>CDSF0903</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>CF gradinita 242</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>03.09.2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>458</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>J-AC 271</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>DALI Cresterea sigurantei rutiere cartier Bucurestii Noi</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>09.09.2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>459</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>J-AC 272</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>DALI Cresterea sigurantei rutiere cartier Piata Romana</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>09.09.2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>460</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>J-AC 273</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>DALI Cresterea sigurantei rutiere cartier Grivita</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>09.09.2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
           <t>461</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr">
+      <c r="B166" t="inlineStr">
         <is>
           <t>J-AC 274</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr">
+      <c r="C166" t="inlineStr">
         <is>
           <t>DALI Cresterea sigurantei rutiere cartier Baneasa</t>
         </is>
       </c>
-      <c r="D159" t="inlineStr">
+      <c r="D166" t="inlineStr">
         <is>
           <t>09.09.2025</t>
         </is>

</xml_diff>

<commit_message>
Update report generation to include Wrike project names and refresh report timestamps
</commit_message>
<xml_diff>
--- a/extrase_pt_conta.xlsx
+++ b/extrase_pt_conta.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D166"/>
+  <dimension ref="A1:E166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,10 +433,15 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Nume Proiect</t>
+          <t>Nume Proiect (Registru)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
+        <is>
+          <t>Nume Proiect (Wrike)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
         <is>
           <t>Data Contract</t>
         </is>
@@ -460,6 +465,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Cheia 1: Panouri fotovoltaice pe cladiri publice - scoli</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>22.02.2024</t>
         </is>
       </c>
@@ -482,6 +492,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Asist clarificari Ef Energ PRBI</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>04.11.2025</t>
         </is>
       </c>
@@ -504,6 +519,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>BUZĂU - SF PT CAMPUS</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>30.06.2025</t>
         </is>
       </c>
@@ -526,6 +546,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>CONSTANTA - PT CAV</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>07.05.2025</t>
         </is>
       </c>
@@ -548,6 +573,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>BUCURESTI ASB - SF CCTV</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>13.11.2025</t>
         </is>
       </c>
@@ -570,6 +600,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>SPITAL PALIATIE PLOIESTI</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>13.05.2025</t>
         </is>
       </c>
@@ -592,6 +627,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>Gradinita nr 1 MP</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>13.06.2025</t>
         </is>
       </c>
@@ -614,6 +654,11 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>Colegiul Elena Doamna MP</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>13.06.2025</t>
         </is>
       </c>
@@ -636,6 +681,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>BUZAU - DALI Pasaj Nehoiasu</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>04.06.2024</t>
         </is>
       </c>
@@ -658,6 +708,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>BUFTEA - DALI DTAC GRADINITA</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>04.08.2025</t>
         </is>
       </c>
@@ -680,6 +735,11 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
+          <t>UMF - SF DTAC - C1</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
           <t>07.05.2025</t>
         </is>
       </c>
@@ -702,6 +762,11 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>BUFTEA - DALI DTAC SCOALA NR. 2</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>04.08.2025</t>
         </is>
       </c>
@@ -724,6 +789,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
+          <t>SIBIU - STUDIU DE TRAFIC SURA MARE</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>17.06.2024</t>
         </is>
       </c>
@@ -746,6 +816,11 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
+          <t>CALARASI - DNSH REABILITARE BRAT BORCEA</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
           <t>17.06.2025</t>
         </is>
       </c>
@@ -768,6 +843,11 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
+          <t>Spital HOREZU</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>05.12.2024</t>
         </is>
       </c>
@@ -790,6 +870,11 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
+          <t>CONSTANTA - Actualizare ST AUTOBAZĂ (&amp; SO AUTOBUZE)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>20.06.2025</t>
         </is>
       </c>
@@ -812,6 +897,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
+          <t>SECTOR 5 - SO Statii Autobuz</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
           <t>28.05.2024</t>
         </is>
       </c>
@@ -834,6 +924,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
+          <t>SF CAV CONSTANȚA (Mare)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
           <t>19.06.2023</t>
         </is>
       </c>
@@ -856,6 +951,11 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
+          <t>CONSULTANTA EFICIENTA ENERGETICA CLADIRI MUZEU NZEB 3.3</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
           <t>01.04.2025</t>
         </is>
       </c>
@@ -878,6 +978,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
+          <t>CALARASI - SF PT ITS</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
           <t>29.11.2023</t>
         </is>
       </c>
@@ -900,6 +1005,11 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
+          <t>CORIDOR MOBILITATE PRSE</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
           <t>17.02.2025</t>
         </is>
       </c>
@@ -922,6 +1032,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
+          <t>CAMPINA - SF ITS 1 DIGITALIZARE</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
           <t>20.03.2023</t>
         </is>
       </c>
@@ -944,6 +1059,11 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
+          <t>PIATRA NEAMT - DTAC+PT Modificare POAT</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
           <t>15.10.2025</t>
         </is>
       </c>
@@ -966,6 +1086,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
+          <t>Camin internat C16 MP</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
           <t>15.07.2025</t>
         </is>
       </c>
@@ -988,6 +1113,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
+          <t>BUZAU - PMUD - GIS</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
           <t>25.07.2023</t>
         </is>
       </c>
@@ -1010,6 +1140,11 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
+          <t>CONSTANTA - SF PT Autobaza</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
           <t>07.07.2023</t>
         </is>
       </c>
@@ -1032,6 +1167,11 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
+          <t>BUZAU - SF E-TRUCK</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
           <t>03.09.2025</t>
         </is>
       </c>
@@ -1054,6 +1194,11 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
+          <t>Sector 5 - Treceri de pietoni suprainaltate</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
           <t>12.03.2025</t>
         </is>
       </c>
@@ -1076,6 +1221,11 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
+          <t>BUZAU - DALI PASAJ DRAGAICA</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
           <t>19.09.2025</t>
         </is>
       </c>
@@ -1098,6 +1248,11 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
+          <t>CALARASI POAT DALI PT Mobilitate</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
           <t>01.03.2022</t>
         </is>
       </c>
@@ -1120,6 +1275,11 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
+          <t>PRJ 1 - EXTRACTION</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
           <t>20.08.2024</t>
         </is>
       </c>
@@ -1140,7 +1300,12 @@
           <t>Consultanta accesare fonduri</t>
         </is>
       </c>
-      <c r="D33" s="1" t="n">
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>SERVICII COMUNITARE DGASPC S5 PIDS</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="n">
         <v>45483</v>
       </c>
     </row>
@@ -1162,6 +1327,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
+          <t>Muntii Carpati - Centre multifunctionale DGASPC S5 PIDS</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
           <t>14.11.2024</t>
         </is>
       </c>
@@ -1184,6 +1354,11 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
+          <t>DGASPC Sector 5 - Panouri fotovoltaice AFM</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
           <t>10.06.2024</t>
         </is>
       </c>
@@ -1206,6 +1381,11 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
+          <t>Continuare lucrări reabilitare corp clădire Grădinița nr. 269 modificare de temă și finalizare lucrări</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
           <t>05.03.2024</t>
         </is>
       </c>
@@ -1228,6 +1408,11 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
+          <t>Sector 5 - DTAD 13 SEPTEMBRIE</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
           <t>24.06.2025</t>
         </is>
       </c>
@@ -1250,6 +1435,11 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
+          <t>GIURGIU- SF CENTRU INTEGRAT</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
           <t>16.05.2022</t>
         </is>
       </c>
@@ -1272,6 +1462,11 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
+          <t>CALARASI STUDII DNSH</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
           <t>26.09.2024</t>
         </is>
       </c>
@@ -1294,6 +1489,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
+          <t>PUZ - CAV ADI Bucuresti</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
           <t>17.10.2023</t>
         </is>
       </c>
@@ -1316,6 +1516,11 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
+          <t>BUCUREȘTI SECTOR 3 - PARC PANTELIMON</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
           <t>08.05.2025</t>
         </is>
       </c>
@@ -1338,6 +1543,11 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
+          <t>SECTOR 5 - DTAC PT nZEB Tineri</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
           <t>30.06.2025</t>
         </is>
       </c>
@@ -1360,6 +1570,11 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
+          <t>CONSTANȚA - DALI PT - Inel 2</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
           <t>02.08.2021</t>
         </is>
       </c>
@@ -1382,6 +1597,11 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
+          <t>BUZAU - STUDIU DE TRAFIC PASAJ</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
           <t>30.08.2024</t>
         </is>
       </c>
@@ -1404,6 +1624,11 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
+          <t>BOTOSANI - SF CENTRU INTEGRAT</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
           <t>06.06.2023</t>
         </is>
       </c>
@@ -1426,6 +1651,11 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
+          <t>BOTOSANI - SF Statii Transport Public</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
           <t>06.06.2023</t>
         </is>
       </c>
@@ -1448,6 +1678,11 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
+          <t>GALATI - STUDIU DE TRAFIC</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
           <t>07.08.2024</t>
         </is>
       </c>
@@ -1470,6 +1705,11 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
+          <t>MP PNRR - CAMPINA (ITS1)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
           <t>06.04.2023</t>
         </is>
       </c>
@@ -1492,6 +1732,11 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
+          <t>CALARASI - STUDIU DE TRAFIC</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
           <t>22.10.2024</t>
         </is>
       </c>
@@ -1514,6 +1759,11 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
+          <t>CALARASI - ACTUALIZARE POAT Mobilitate</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
           <t>22.10.2024</t>
         </is>
       </c>
@@ -1536,6 +1786,11 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
+          <t>CĂLĂRAȘI - POAT - REGENERARE URBANĂ CARTIERE - ACTUALIZARE</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
           <t>22.10.2024</t>
         </is>
       </c>
@@ -1558,6 +1813,11 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
+          <t>MP G269 PRBI</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
           <t>28.08.2025</t>
         </is>
       </c>
@@ -1580,6 +1840,11 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
+          <t>PLOIESTI - REGENERARE PARAUL DAMBU</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
           <t>06.08.2025</t>
         </is>
       </c>
@@ -1602,6 +1867,11 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
+          <t>BUZĂU- SF PT POAT HUB</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
           <t>01.11.2021</t>
         </is>
       </c>
@@ -1624,6 +1894,11 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
+          <t>Eficienta energetica blocuri - ETAPA 3 (CTR 165 172800)</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
           <t>22.06.2023</t>
         </is>
       </c>
@@ -1646,6 +1921,11 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
+          <t>Eficienta energetica blocuri - ETAPA 4 (CTR 166 172803)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
           <t>22.06.2023</t>
         </is>
       </c>
@@ -1668,6 +1948,11 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
+          <t>Eficienta energetica blocuri - ETAPA 1 (CTR 167 172807)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
           <t>22.06.2023</t>
         </is>
       </c>
@@ -1690,6 +1975,11 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
+          <t>ALBA IULIA - SF PT AT - Sistem de ticketing</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
           <t>13.02.2025</t>
         </is>
       </c>
@@ -1712,6 +2002,11 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
+          <t>TPBI - SF Sistem de informare călători</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
           <t>09.12.2025</t>
         </is>
       </c>
@@ -1734,6 +2029,11 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
+          <t>Eficienta energetica blocuri - ETAPA 2 (CTR 168 172809)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
           <t>22.06.2023</t>
         </is>
       </c>
@@ -1756,6 +2056,11 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
+          <t>ROȘIORII DE VEDE - REGENERARE URBANĂ PARC GRĂDINĂ PUBLICĂ</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
           <t>14.10.2024</t>
         </is>
       </c>
@@ -1778,6 +2083,11 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
+          <t>BUFTEA - DALI Suprainaltate</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
           <t>23.12.205</t>
         </is>
       </c>
@@ -1800,6 +2110,11 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
+          <t>Strategie M100 Galati + CF</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
           <t>04.09.2024</t>
         </is>
       </c>
@@ -1822,6 +2137,11 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
+          <t>BUCURESTI - SECTOR 5 - PT STATII INCARCARE</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
           <t>09.10.2025</t>
         </is>
       </c>
@@ -1844,6 +2164,11 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
+          <t>SECTOR 5 - SO Asistent virtual</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
           <t>30.08.2024</t>
         </is>
       </c>
@@ -1866,6 +2191,11 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
+          <t>FOCSANI - SF PT Coridor Nord - Sud</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
           <t>18.02.2022</t>
         </is>
       </c>
@@ -1888,6 +2218,11 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
+          <t>BUZĂU - PLAN INTEGRAT DE REGENERARE URBANA_1</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
           <t>03.10.2024</t>
         </is>
       </c>
@@ -1910,6 +2245,11 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
+          <t>BUZAU - SO TRANSPORT PUBLIC - AUTOBUZE</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
           <t>20.10.2023</t>
         </is>
       </c>
@@ -1932,6 +2272,11 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
+          <t>BUZAU - SO TRANSPORT PUBLIC - MICROBUZE</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
           <t>27.10.2023</t>
         </is>
       </c>
@@ -1954,6 +2299,11 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
+          <t>PRJ 2 - PROCESSING &amp; RECYCLING</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
           <t>24.10.2025</t>
         </is>
       </c>
@@ -1976,6 +2326,11 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
+          <t>GALATI MP DEPOU</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
           <t>13.10.2025</t>
         </is>
       </c>
@@ -1998,6 +2353,11 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
+          <t>TECUCI - DTAC PT ITS</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
           <t>27.03.2024</t>
         </is>
       </c>
@@ -2020,6 +2380,11 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
+          <t>CF DAMBU</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
           <t>22.09.2025</t>
         </is>
       </c>
@@ -2042,6 +2407,11 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
+          <t>FONDUL LOCAL PNRR C10</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
           <t>13.09.2022</t>
         </is>
       </c>
@@ -2064,6 +2434,11 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
+          <t>BUZAU - SO PLATFORMA ELECTRONICA MaaS</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
           <t>13.11.2023</t>
         </is>
       </c>
@@ -2086,6 +2461,11 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
+          <t>BUZAU - SO Delegare transport public 2025</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
           <t>30.06.2025</t>
         </is>
       </c>
@@ -2108,6 +2488,11 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
+          <t>HOREZU - PT MOBILITATE</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
           <t>28.08.2025</t>
         </is>
       </c>
@@ -2130,6 +2515,11 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
+          <t>CHIȘINĂU - STUDIU DE E-TICKETING</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
           <t>11.12.2023</t>
         </is>
       </c>
@@ -2152,6 +2542,11 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
+          <t>CONSTANTA - SF STATII INCARCARE</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
           <t>23.10.2024</t>
         </is>
       </c>
@@ -2174,6 +2569,11 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
+          <t>GALATI MP INFRASTRUCTURA</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
           <t>03.11.2025</t>
         </is>
       </c>
@@ -2196,6 +2596,11 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
+          <t>Functionar Public Virtual (GIS SITE CARTOGRAFIERE)</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
           <t>10.12.2024</t>
         </is>
       </c>
@@ -2218,6 +2623,11 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
+          <t>CALIMANESTI - ACTUALIZARE SO DELEGARE TP</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
           <t>05.12.2024</t>
         </is>
       </c>
@@ -2240,6 +2650,11 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
+          <t>BUZĂU - SF PARCĂRI SUPRATERANE</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
           <t>21.11.2022</t>
         </is>
       </c>
@@ -2262,6 +2677,11 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
+          <t>ROSIORII DE VEDE - SF-TIC</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
           <t>20.12.2024</t>
         </is>
       </c>
@@ -2284,6 +2704,11 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
+          <t>DROBETA - SF ITS</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
           <t>06.06.2023</t>
         </is>
       </c>
@@ -2306,6 +2731,11 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
+          <t>CAMPINA - SO DELEGARE TP</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
           <t>26.05.2025</t>
         </is>
       </c>
@@ -2328,6 +2758,11 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
+          <t>CF HUB Buzau PRSE Mob</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
           <t>23.12.2024</t>
         </is>
       </c>
@@ -2350,6 +2785,11 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
+          <t>PT CAV BUZAU</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
           <t>30.12.2024</t>
         </is>
       </c>
@@ -2372,6 +2812,11 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
+          <t>TECUCI- SF TRAFIC MANAGEMENT</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
           <t>08.05.2023</t>
         </is>
       </c>
@@ -2394,6 +2839,11 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
+          <t>CF Servicii ingrijiri la domiciliu varstnici PIDS Magurele</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
           <t>28.08.2025</t>
         </is>
       </c>
@@ -2416,6 +2866,11 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
+          <t>CF PNCCRS PRBI</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
           <t>17.07.2025</t>
         </is>
       </c>
@@ -2438,6 +2893,11 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
+          <t>MP PNRR - CAMPINA (bus)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
           <t>29.05.2023</t>
         </is>
       </c>
@@ -2460,6 +2920,11 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
+          <t>PISTE PRBI</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
           <t>02.09.2025</t>
         </is>
       </c>
@@ -2482,6 +2947,11 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
+          <t>AFM CLADIRI PUBLICE - Scoala 143</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
           <t>07.09.2023</t>
         </is>
       </c>
@@ -2504,6 +2974,11 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
+          <t>TARGOVISTE - SF ITS 1</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
           <t>27.07.2023</t>
         </is>
       </c>
@@ -2526,6 +3001,11 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
+          <t>TARGOVISTE - SF ITS 2</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
           <t>27.07.2023</t>
         </is>
       </c>
@@ -2548,6 +3028,11 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
+          <t>DNSH - PR BI Blocuri - Ef. Energ</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
           <t>26.09.2023</t>
         </is>
       </c>
@@ -2570,6 +3055,11 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
+          <t>HOREZU- SF POR</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
           <t>02.02.2024</t>
         </is>
       </c>
@@ -2592,6 +3082,11 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
+          <t>Modernizarea Serviciului de Transport Persoane din orasul Horezu judetul Valcea</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
           <t>02.02.2024</t>
         </is>
       </c>
@@ -2614,6 +3109,11 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
+          <t>REGHIN - SF ITS</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
           <t>08.08.2024</t>
         </is>
       </c>
@@ -2636,6 +3136,11 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
+          <t>DNSH - PR - GRADINITA 269</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
           <t>20.03.2024</t>
         </is>
       </c>
@@ -2658,6 +3163,11 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
+          <t>SUCEAVA - SF PT TP ETAPA 2</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
           <t>01.08.2022</t>
         </is>
       </c>
@@ -2680,6 +3190,11 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
+          <t>SF CAV BRAȘOV (Mare)</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
           <t>15.09.2023</t>
         </is>
       </c>
@@ -2702,6 +3217,11 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
+          <t>BRAILA - SO &amp; ST</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
           <t>03.12.2024</t>
         </is>
       </c>
@@ -2724,6 +3244,11 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
+          <t>BOTOSANI - CONST TEHN - EXPERT COOPTAT - Autobuze PNRR</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
           <t>05.02.2024</t>
         </is>
       </c>
@@ -2746,6 +3271,11 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
+          <t>TULCEA - DTAC PT - ITS + AUTOBAZA</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
           <t>25.07.2024</t>
         </is>
       </c>
@@ -2768,6 +3298,11 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
+          <t>BACAU - DTAC+PT CAMPUS</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
           <t>07.07.2025</t>
         </is>
       </c>
@@ -2790,6 +3325,11 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
+          <t>CAMPINA - SF PT AUTOBAZA</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
           <t>18.07.2025</t>
         </is>
       </c>
@@ -2812,6 +3352,11 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
+          <t>CNAB - DALI MODERNIZARE HVAC AIHCB</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
           <t>23.01.2025</t>
         </is>
       </c>
@@ -2834,6 +3379,11 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
+          <t>UMF - PT Corp cladire C2</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
           <t>06.12.2024</t>
         </is>
       </c>
@@ -2856,6 +3406,11 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
+          <t>PITESTI - SO AUTOBUZE</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
           <t>26.05.2023</t>
         </is>
       </c>
@@ -2878,6 +3433,11 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
+          <t>DROBETA - DTAC DTOE PT ITS 1</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
           <t>06.08.2024</t>
         </is>
       </c>
@@ -2900,6 +3460,11 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
+          <t>Consultari NEB - Fort 13</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
           <t>05.11.2025</t>
         </is>
       </c>
@@ -2922,6 +3487,11 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
+          <t>CF AUTOBAZA PRSM</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
           <t>06.08.2025</t>
         </is>
       </c>
@@ -2944,6 +3514,11 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
+          <t>SUCEAVA - SF PT ITS STATII</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
           <t>12.09.2022</t>
         </is>
       </c>
@@ -2966,6 +3541,11 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
+          <t>UMF - SF Corp cladire C2</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
           <t>15.11.2024</t>
         </is>
       </c>
@@ -2988,6 +3568,11 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
+          <t>ALEXANDRIA DALI Pietonal</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
           <t>12.07.2023</t>
         </is>
       </c>
@@ -3010,6 +3595,11 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
+          <t>MP PNRR - CAMPINA (ITS2)</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
           <t>01.09.2023</t>
         </is>
       </c>
@@ -3032,6 +3622,11 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
+          <t>DROBETA - DALI PT POAT MOBILITATE</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
           <t>06.10.2022</t>
         </is>
       </c>
@@ -3054,6 +3649,11 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
+          <t>CONSTANTA - PT DTAC DE ATH - ZONA CENTRALA - REST LUCRARI</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
           <t>19.02.2025</t>
         </is>
       </c>
@@ -3076,6 +3676,11 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
+          <t>CONSULTARE NEB - PARC PANTELIMON 7.1 7.3</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
           <t>04.02.2025</t>
         </is>
       </c>
@@ -3098,6 +3703,11 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
+          <t>CONSULTARE NEB - NENITESCU 7.2</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
           <t>04.02.2025</t>
         </is>
       </c>
@@ -3120,6 +3730,11 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
+          <t>CAMPINA - SF ITS 2</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
           <t>28.09.2023</t>
         </is>
       </c>
@@ -3142,6 +3757,11 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
+          <t>CONSTANTA POAT PRSE</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
           <t>25.02.2025</t>
         </is>
       </c>
@@ -3164,6 +3784,11 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
+          <t>Baia de Aries - ITS</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
           <t>07.07.2025</t>
         </is>
       </c>
@@ -3186,6 +3811,11 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
+          <t>MP POR 14-20 DEVA autobuze</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
           <t>16.06.2020</t>
         </is>
       </c>
@@ -3208,6 +3838,11 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
+          <t>CONSTANȚA - Greener Cities</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
           <t>26.02.2026</t>
         </is>
       </c>
@@ -3230,6 +3865,11 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
+          <t>SF CAV BRAȘOV (Mic)</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
           <t>13.03.2023</t>
         </is>
       </c>
@@ -3252,6 +3892,11 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
+          <t>BOTOSANI - PT+EXEC CENTRU INTEGRAT</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
           <t>27.02.2025</t>
         </is>
       </c>
@@ -3274,6 +3919,11 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
+          <t>SECTOR 1 - DTAC PT Suprainaltate Bucurestii Noi</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
           <t>21.02.2023</t>
         </is>
       </c>
@@ -3296,6 +3946,11 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
+          <t>Consultanta cladiri Bauhaus Inst Pneuftiziologie Marius Nasta - corp nou</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
           <t>09.04.2025</t>
         </is>
       </c>
@@ -3318,6 +3973,11 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
+          <t>MP PNRR - SECTOR 5 (dotari)</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
           <t>08.04.2024</t>
         </is>
       </c>
@@ -3340,6 +4000,11 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
+          <t>Actualizare SIDU HOREZU 2021-2027</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
           <t>05.03.2024</t>
         </is>
       </c>
@@ -3362,6 +4027,11 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
+          <t>MP PNRR - CONSTANTA (bus)</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
           <t>17.03.2023</t>
         </is>
       </c>
@@ -3384,6 +4054,11 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
+          <t>ASB - DALI + DTAC REABILITARE SEDIU</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
           <t>26.06.2025</t>
         </is>
       </c>
@@ -3406,6 +4081,11 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
+          <t>ALBA IULIA - SF Ticketing</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
           <t>21.01.2025</t>
         </is>
       </c>
@@ -3428,6 +4108,11 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
+          <t>MP PNRR - SUCEAVA (autobuze)</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
           <t>15.02.2023</t>
         </is>
       </c>
@@ -3450,6 +4135,11 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
+          <t>SOCEP - SF Terminal intermodal</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
           <t>10.02.2025</t>
         </is>
       </c>
@@ -3472,6 +4162,11 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
+          <t>ALBA IULIA - SF PT AT - Sistem de afisaj</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
           <t>05.06.2025</t>
         </is>
       </c>
@@ -3494,6 +4189,11 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
+          <t>HOREZU- SF cu el DALI SPITAL</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
           <t>01.08.2024</t>
         </is>
       </c>
@@ -3516,6 +4216,11 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
+          <t>BOTOSANI - CS Autobuze PNRR</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
           <t>13.03.2023</t>
         </is>
       </c>
@@ -3538,6 +4243,11 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
+          <t>BUZAU - SF CITY AIR</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
           <t>19.04.2024</t>
         </is>
       </c>
@@ -3560,6 +4270,11 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
+          <t>GALATI - DALI GRADINA DE VARA</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
           <t>16.01.2025</t>
         </is>
       </c>
@@ -3582,6 +4297,11 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
+          <t>EXPERTIZE TEHNICE SCOALA 126&amp;103</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
           <t>29.04.2025</t>
         </is>
       </c>
@@ -3604,6 +4324,11 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
+          <t>MP POR 14-20 IASI ticketing</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
           <t>12.08.2020</t>
         </is>
       </c>
@@ -3626,6 +4351,11 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
+          <t>MP PNRR - SUCEAVA (ITS)</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
           <t>01.03.2023</t>
         </is>
       </c>
@@ -3648,6 +4378,11 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
+          <t>BUCURESTI - SISTEM ITS SMART&amp;GREEN Mobility</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
           <t>27.10.2023</t>
         </is>
       </c>
@@ -3670,6 +4405,11 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
+          <t>BUFTEA - SO ST AUTOBUZE</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
           <t>04.07.2025</t>
         </is>
       </c>
@@ -3692,6 +4432,11 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
+          <t>BUFTEA - SF AUTOBAZA</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
           <t>04.07.2025</t>
         </is>
       </c>
@@ -3714,6 +4459,11 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
+          <t>SUCEAVA - CS Autobuze PNRR</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
           <t>08.03.2022</t>
         </is>
       </c>
@@ -3736,6 +4486,11 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
+          <t>HOREZU - SF CU ELEMENTE DE DALI - SPITAL</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
           <t>05.09.2025</t>
         </is>
       </c>
@@ -3758,6 +4513,11 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
+          <t>CRAIOVA - AEROPORT</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
           <t>17.12.2024</t>
         </is>
       </c>
@@ -3780,6 +4540,11 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
+          <t>SO CENTRU COMERCIAL</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
           <t>02.10.2025</t>
         </is>
       </c>
@@ -3802,6 +4567,11 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
+          <t>FOCȘANI - DALI REABILITARE SI REGENERARE ZONA PARC TEATRU</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
           <t>02.10.2025</t>
         </is>
       </c>
@@ -3824,6 +4594,11 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
+          <t>AMENAJAREA SCUARULUI DE LA INTERSECȚIA STRĂZILOR CALEA DOROBANȚI CU STRADA RADU BELLER</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
           <t>30.12.2024</t>
         </is>
       </c>
@@ -3846,6 +4621,11 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
+          <t>FOCȘANI - DALI REGENERARE URBANĂ A ZONEI CENTRALE A MUNICIPIULUI FOCȘANI</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
           <t>22.10.2025</t>
         </is>
       </c>
@@ -3868,6 +4648,11 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
+          <t>CONSULTANTA REGENERARE URBANA IOR 7.1 7.3</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
           <t>20.03.2025</t>
         </is>
       </c>
@@ -3890,6 +4675,11 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
+          <t>PLOIESTI - SF DTAC SPITAL</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
           <t>12.05.2025</t>
         </is>
       </c>
@@ -3912,6 +4702,11 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
+          <t>BUCURESTI - STUDIU DE TRAFIC - UNIRII</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
           <t>26.02.2024</t>
         </is>
       </c>
@@ -3934,6 +4729,11 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
+          <t>BUCURESTI - DTAC PT Relocare troleibuz Unirii</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
           <t>30.04.2024</t>
         </is>
       </c>
@@ -3956,6 +4756,11 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
+          <t>BUCURESTI - STUDIU DE TRAFIC - UNIRII E2</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
           <t>30.04.2024</t>
         </is>
       </c>
@@ -3978,6 +4783,11 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
+          <t>CF S5 G242</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
           <t>03.09.2025</t>
         </is>
       </c>
@@ -4000,6 +4810,11 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
+          <t>SECTOR 1 - DALI Suprainaltate Bucurestii Noi</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
           <t>09.09.2025</t>
         </is>
       </c>
@@ -4022,6 +4837,11 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
+          <t>SECTOR 1 - DALI Suprainaltate Romana</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
           <t>09.09.2025</t>
         </is>
       </c>
@@ -4044,6 +4864,11 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
+          <t>SECTOR 1 - DALI Suprainaltate Grivita</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
           <t>09.09.2025</t>
         </is>
       </c>
@@ -4065,6 +4890,11 @@
         </is>
       </c>
       <c r="D166" t="inlineStr">
+        <is>
+          <t>SECTOR 1 - DALI Suprainaltate Baneasa</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
         <is>
           <t>09.09.2025</t>
         </is>

</xml_diff>